<commit_message>
Add 13 AYCE-Wagyu hybrid places (yakiniku/shabu/AYCE-sushi) with format tag
These are the dedicated AYCE-Wagyu programs that the omakase research missed —
they're the actual reality of NYC's 'unlimited wagyu' category. Tagged with
format='ayce_wagyu_hybrid' so they don't get confused with counter omakase.

- Dataset 188 -> 201 restaurants (188 omakase + 13 hybrids)
- 20 AYCE-Wagyu offerings total (7 omakase + 13 hybrids)
- New Format filter (Omakase only / Hybrid only / All)
- 'Yakiniku' badge in restaurant name column for hybrid entries
- Legend explains the hybrid format
- step3 now merges specialty data from hybrid file too
- step3 propagates format field through scored output

Hybrid AYCE-Wagyu programs added:
- Wagyu Place (Flushing), Niku X (Midtown), Mikiya x2, Chubby Cattle (SoHo),
  Y Space (Flushing), Wagyu Yama (Flushing), Hiyake x2, Gyu-Ichiro,
  Nikushou Sakai (Flushing), Umiya LIC, Asuka (Chelsea)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Omakase_Ratings.xlsx
+++ b/Omakase_Ratings.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P189"/>
+  <dimension ref="A1:P202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -587,13 +587,13 @@
         <v>4.107</v>
       </c>
       <c r="L2" t="n">
-        <v>32.6</v>
+        <v>32</v>
       </c>
       <c r="M2" t="n">
         <v>4.061</v>
       </c>
       <c r="N2" t="n">
-        <v>30.8</v>
+        <v>29.3</v>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
@@ -639,13 +639,13 @@
         <v>3.545</v>
       </c>
       <c r="L3" t="n">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="M3" t="n">
         <v>3.563</v>
       </c>
       <c r="N3" t="n">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
@@ -691,13 +691,13 @@
         <v>4.143</v>
       </c>
       <c r="L4" t="n">
-        <v>40.1</v>
+        <v>39</v>
       </c>
       <c r="M4" t="n">
         <v>4.143</v>
       </c>
       <c r="N4" t="n">
-        <v>40</v>
+        <v>37.9</v>
       </c>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
@@ -739,13 +739,13 @@
         <v>3.86</v>
       </c>
       <c r="L5" t="n">
-        <v>6.4</v>
+        <v>7</v>
       </c>
       <c r="M5" t="n">
         <v>3.88</v>
       </c>
       <c r="N5" t="n">
-        <v>18.9</v>
+        <v>18.2</v>
       </c>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
@@ -787,13 +787,13 @@
         <v>3.958</v>
       </c>
       <c r="L6" t="n">
-        <v>19.3</v>
+        <v>19.5</v>
       </c>
       <c r="M6" t="n">
         <v>3.886</v>
       </c>
       <c r="N6" t="n">
-        <v>21.1</v>
+        <v>20.2</v>
       </c>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
@@ -835,13 +835,13 @@
         <v>4.324</v>
       </c>
       <c r="L7" t="n">
-        <v>74.90000000000001</v>
+        <v>72.5</v>
       </c>
       <c r="M7" t="n">
         <v>4.152</v>
       </c>
       <c r="N7" t="n">
-        <v>40.5</v>
+        <v>38.4</v>
       </c>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
@@ -887,13 +887,13 @@
         <v>4.25</v>
       </c>
       <c r="L8" t="n">
-        <v>53.5</v>
+        <v>52</v>
       </c>
       <c r="M8" t="n">
         <v>4.3</v>
       </c>
       <c r="N8" t="n">
-        <v>59.5</v>
+        <v>57.1</v>
       </c>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
@@ -939,13 +939,13 @@
         <v>4.234</v>
       </c>
       <c r="L9" t="n">
-        <v>51.3</v>
+        <v>50</v>
       </c>
       <c r="M9" t="n">
         <v>4.776</v>
       </c>
       <c r="N9" t="n">
-        <v>98.90000000000001</v>
+        <v>97</v>
       </c>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
@@ -1013,13 +1013,13 @@
         <v>3.865</v>
       </c>
       <c r="L11" t="n">
-        <v>7.5</v>
+        <v>8</v>
       </c>
       <c r="M11" t="n">
         <v>3.957</v>
       </c>
       <c r="N11" t="n">
-        <v>24.9</v>
+        <v>23.7</v>
       </c>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
@@ -1061,13 +1061,13 @@
         <v>4.389</v>
       </c>
       <c r="L12" t="n">
-        <v>85.59999999999999</v>
+        <v>83</v>
       </c>
       <c r="M12" t="n">
         <v>4.445</v>
       </c>
       <c r="N12" t="n">
-        <v>77.3</v>
+        <v>73.7</v>
       </c>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr">
@@ -1113,13 +1113,13 @@
         <v>4.33</v>
       </c>
       <c r="L13" t="n">
-        <v>76.5</v>
+        <v>74</v>
       </c>
       <c r="M13" t="n">
         <v>4.309</v>
       </c>
       <c r="N13" t="n">
-        <v>60</v>
+        <v>57.6</v>
       </c>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr">
@@ -1165,13 +1165,13 @@
         <v>4.296</v>
       </c>
       <c r="L14" t="n">
-        <v>68.40000000000001</v>
+        <v>66.5</v>
       </c>
       <c r="M14" t="n">
         <v>4.465</v>
       </c>
       <c r="N14" t="n">
-        <v>80.5</v>
+        <v>76.8</v>
       </c>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
@@ -1217,13 +1217,13 @@
         <v>4.078</v>
       </c>
       <c r="L15" t="n">
-        <v>28.9</v>
+        <v>28.5</v>
       </c>
       <c r="M15" t="n">
         <v>4.078</v>
       </c>
       <c r="N15" t="n">
-        <v>33</v>
+        <v>31.3</v>
       </c>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
@@ -1269,13 +1269,13 @@
         <v>4.336</v>
       </c>
       <c r="L16" t="n">
-        <v>77.5</v>
+        <v>75</v>
       </c>
       <c r="M16" t="n">
         <v>4.276</v>
       </c>
       <c r="N16" t="n">
-        <v>56.8</v>
+        <v>54.5</v>
       </c>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
@@ -1317,13 +1317,13 @@
         <v>4.042</v>
       </c>
       <c r="L17" t="n">
-        <v>26.7</v>
+        <v>26.5</v>
       </c>
       <c r="M17" t="n">
         <v>4.201</v>
       </c>
       <c r="N17" t="n">
-        <v>47</v>
+        <v>44.9</v>
       </c>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr">
@@ -1369,13 +1369,13 @@
         <v>4.092</v>
       </c>
       <c r="L18" t="n">
-        <v>30.5</v>
+        <v>30</v>
       </c>
       <c r="M18" t="n">
         <v>3.881</v>
       </c>
       <c r="N18" t="n">
-        <v>20</v>
+        <v>19.2</v>
       </c>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr">
@@ -1417,13 +1417,13 @@
         <v>4.252</v>
       </c>
       <c r="L19" t="n">
-        <v>54.5</v>
+        <v>53</v>
       </c>
       <c r="M19" t="n">
         <v>4.212</v>
       </c>
       <c r="N19" t="n">
-        <v>48.1</v>
+        <v>46.5</v>
       </c>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr">
@@ -1469,13 +1469,13 @@
         <v>3.985</v>
       </c>
       <c r="L20" t="n">
-        <v>21.9</v>
+        <v>22</v>
       </c>
       <c r="M20" t="n">
         <v>3.827</v>
       </c>
       <c r="N20" t="n">
-        <v>13</v>
+        <v>12.6</v>
       </c>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
@@ -1521,13 +1521,13 @@
         <v>4.387</v>
       </c>
       <c r="L21" t="n">
-        <v>85</v>
+        <v>82.5</v>
       </c>
       <c r="M21" t="n">
         <v>4.649</v>
       </c>
       <c r="N21" t="n">
-        <v>95.7</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr">
@@ -1565,13 +1565,13 @@
         <v>4.095</v>
       </c>
       <c r="L22" t="n">
-        <v>31</v>
+        <v>30.5</v>
       </c>
       <c r="M22" t="n">
         <v>4.116</v>
       </c>
       <c r="N22" t="n">
-        <v>36.8</v>
+        <v>34.8</v>
       </c>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
@@ -1617,13 +1617,13 @@
         <v>4.544</v>
       </c>
       <c r="L23" t="n">
-        <v>95.7</v>
+        <v>95</v>
       </c>
       <c r="M23" t="n">
         <v>4.509</v>
       </c>
       <c r="N23" t="n">
-        <v>85.40000000000001</v>
+        <v>81.3</v>
       </c>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr">
@@ -1669,13 +1669,13 @@
         <v>4.142</v>
       </c>
       <c r="L24" t="n">
-        <v>39.6</v>
+        <v>38.5</v>
       </c>
       <c r="M24" t="n">
         <v>4.142</v>
       </c>
       <c r="N24" t="n">
-        <v>39.5</v>
+        <v>37.4</v>
       </c>
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
@@ -1721,13 +1721,13 @@
         <v>4.636</v>
       </c>
       <c r="L25" t="n">
-        <v>97.90000000000001</v>
+        <v>97</v>
       </c>
       <c r="M25" t="n">
         <v>4.69</v>
       </c>
       <c r="N25" t="n">
-        <v>97.3</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr">
@@ -1779,7 +1779,7 @@
         <v>4.045</v>
       </c>
       <c r="N26" t="n">
-        <v>29.7</v>
+        <v>28.3</v>
       </c>
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr">
@@ -1825,13 +1825,13 @@
         <v>4.494</v>
       </c>
       <c r="L27" t="n">
-        <v>94.7</v>
+        <v>94</v>
       </c>
       <c r="M27" t="n">
         <v>4.378</v>
       </c>
       <c r="N27" t="n">
-        <v>68.09999999999999</v>
+        <v>65.2</v>
       </c>
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr">
@@ -1877,13 +1877,13 @@
         <v>3.982</v>
       </c>
       <c r="L28" t="n">
-        <v>20.9</v>
+        <v>21</v>
       </c>
       <c r="M28" t="n">
         <v>4.191</v>
       </c>
       <c r="N28" t="n">
-        <v>45.4</v>
+        <v>43.4</v>
       </c>
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr">
@@ -1929,13 +1929,13 @@
         <v>4.219</v>
       </c>
       <c r="L29" t="n">
-        <v>49.2</v>
+        <v>48</v>
       </c>
       <c r="M29" t="n">
         <v>4.54</v>
       </c>
       <c r="N29" t="n">
-        <v>87.59999999999999</v>
+        <v>83.3</v>
       </c>
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr">
@@ -1977,13 +1977,13 @@
         <v>3.982</v>
       </c>
       <c r="L30" t="n">
-        <v>20.9</v>
+        <v>21</v>
       </c>
       <c r="M30" t="n">
         <v>4.212</v>
       </c>
       <c r="N30" t="n">
-        <v>48.1</v>
+        <v>46.5</v>
       </c>
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr">
@@ -2029,13 +2029,13 @@
         <v>4.368</v>
       </c>
       <c r="L31" t="n">
-        <v>82.40000000000001</v>
+        <v>80</v>
       </c>
       <c r="M31" t="n">
         <v>4.39</v>
       </c>
       <c r="N31" t="n">
-        <v>69.2</v>
+        <v>66.2</v>
       </c>
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr">
@@ -2081,13 +2081,13 @@
         <v>4.242</v>
       </c>
       <c r="L32" t="n">
-        <v>52.9</v>
+        <v>51.5</v>
       </c>
       <c r="M32" t="n">
         <v>4.479</v>
       </c>
       <c r="N32" t="n">
-        <v>81.59999999999999</v>
+        <v>77.8</v>
       </c>
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr">
@@ -2129,13 +2129,13 @@
         <v>4.554</v>
       </c>
       <c r="L33" s="2" t="n">
-        <v>96.3</v>
+        <v>95.5</v>
       </c>
       <c r="M33" s="2" t="n">
         <v>4.607</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>93</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2174,7 +2174,7 @@
         <v>3.871</v>
       </c>
       <c r="L34" t="n">
-        <v>11.2</v>
+        <v>11.5</v>
       </c>
       <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr">
@@ -2220,13 +2220,13 @@
         <v>4.238</v>
       </c>
       <c r="L35" s="2" t="n">
-        <v>51.9</v>
+        <v>50.5</v>
       </c>
       <c r="M35" s="2" t="n">
         <v>4.398</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>70.8</v>
+        <v>67.7</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2276,13 +2276,13 @@
         <v>4.47</v>
       </c>
       <c r="L36" t="n">
-        <v>92.5</v>
+        <v>91</v>
       </c>
       <c r="M36" t="n">
         <v>4.543</v>
       </c>
       <c r="N36" t="n">
-        <v>88.09999999999999</v>
+        <v>83.8</v>
       </c>
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr">
@@ -2328,13 +2328,13 @@
         <v>4.284</v>
       </c>
       <c r="L37" t="n">
-        <v>65.2</v>
+        <v>63</v>
       </c>
       <c r="M37" t="n">
         <v>4.114</v>
       </c>
       <c r="N37" t="n">
-        <v>36.2</v>
+        <v>34.3</v>
       </c>
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr">
@@ -2377,7 +2377,7 @@
         <v>3.48</v>
       </c>
       <c r="L38" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr">
@@ -2423,13 +2423,13 @@
         <v>4.149</v>
       </c>
       <c r="L39" t="n">
-        <v>41.7</v>
+        <v>40.5</v>
       </c>
       <c r="M39" t="n">
         <v>4.785</v>
       </c>
       <c r="N39" t="n">
-        <v>99.5</v>
+        <v>97.5</v>
       </c>
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr">
@@ -2475,13 +2475,13 @@
         <v>3.865</v>
       </c>
       <c r="L40" t="n">
-        <v>7.5</v>
+        <v>8</v>
       </c>
       <c r="M40" t="n">
         <v>3.881</v>
       </c>
       <c r="N40" t="n">
-        <v>20</v>
+        <v>19.2</v>
       </c>
       <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr">
@@ -2527,13 +2527,13 @@
         <v>4.261</v>
       </c>
       <c r="L41" t="n">
-        <v>56.1</v>
+        <v>54.5</v>
       </c>
       <c r="M41" t="n">
         <v>4.316</v>
       </c>
       <c r="N41" t="n">
-        <v>61.6</v>
+        <v>59.1</v>
       </c>
       <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr">
@@ -2579,13 +2579,13 @@
         <v>3.951</v>
       </c>
       <c r="L42" t="n">
-        <v>18.7</v>
+        <v>19</v>
       </c>
       <c r="M42" t="n">
         <v>3.951</v>
       </c>
       <c r="N42" t="n">
-        <v>24.3</v>
+        <v>23.2</v>
       </c>
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr">
@@ -2627,13 +2627,13 @@
         <v>4.167</v>
       </c>
       <c r="L43" t="n">
-        <v>42.8</v>
+        <v>41.5</v>
       </c>
       <c r="M43" t="n">
         <v>4.188</v>
       </c>
       <c r="N43" t="n">
-        <v>44.3</v>
+        <v>42.4</v>
       </c>
       <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr">
@@ -2685,7 +2685,7 @@
         <v>4.732</v>
       </c>
       <c r="N44" t="n">
-        <v>97.8</v>
+        <v>96</v>
       </c>
       <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr">
@@ -2727,13 +2727,13 @@
         <v>3.869</v>
       </c>
       <c r="L45" t="n">
-        <v>10.2</v>
+        <v>10.5</v>
       </c>
       <c r="M45" t="n">
         <v>3.889</v>
       </c>
       <c r="N45" t="n">
-        <v>21.6</v>
+        <v>20.7</v>
       </c>
       <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr">
@@ -2779,13 +2779,13 @@
         <v>3.913</v>
       </c>
       <c r="L46" t="n">
-        <v>16</v>
+        <v>16.5</v>
       </c>
       <c r="M46" t="n">
         <v>4.027</v>
       </c>
       <c r="N46" t="n">
-        <v>28.6</v>
+        <v>27.3</v>
       </c>
       <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr">
@@ -2831,13 +2831,13 @@
         <v>3.652</v>
       </c>
       <c r="L47" t="n">
-        <v>2.1</v>
+        <v>2.5</v>
       </c>
       <c r="M47" t="n">
         <v>3.843</v>
       </c>
       <c r="N47" t="n">
-        <v>14.6</v>
+        <v>14.1</v>
       </c>
       <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr">
@@ -2879,13 +2879,13 @@
         <v>4.141</v>
       </c>
       <c r="L48" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="M48" t="n">
         <v>4.245</v>
       </c>
       <c r="N48" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr">
@@ -2931,13 +2931,13 @@
         <v>4.583</v>
       </c>
       <c r="L49" t="n">
-        <v>96.8</v>
+        <v>96</v>
       </c>
       <c r="M49" t="n">
         <v>4.756</v>
       </c>
       <c r="N49" t="n">
-        <v>98.40000000000001</v>
+        <v>96.5</v>
       </c>
       <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr">
@@ -2983,13 +2983,13 @@
         <v>3.817</v>
       </c>
       <c r="L50" s="2" t="n">
-        <v>4.8</v>
+        <v>5.5</v>
       </c>
       <c r="M50" s="2" t="n">
         <v>3.825</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>12.4</v>
+        <v>12.1</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3039,13 +3039,13 @@
         <v>4.122</v>
       </c>
       <c r="L51" t="n">
-        <v>35.8</v>
+        <v>35</v>
       </c>
       <c r="M51" t="n">
         <v>4.237</v>
       </c>
       <c r="N51" t="n">
-        <v>51.9</v>
+        <v>50</v>
       </c>
       <c r="O51" t="inlineStr"/>
       <c r="P51" t="inlineStr">
@@ -3091,13 +3091,13 @@
         <v>4.273</v>
       </c>
       <c r="L52" t="n">
-        <v>61.5</v>
+        <v>59.5</v>
       </c>
       <c r="M52" t="n">
         <v>4.461</v>
       </c>
       <c r="N52" t="n">
-        <v>79.5</v>
+        <v>75.8</v>
       </c>
       <c r="O52" t="inlineStr"/>
       <c r="P52" t="inlineStr">
@@ -3143,13 +3143,13 @@
         <v>4.345</v>
       </c>
       <c r="L53" t="n">
-        <v>78.09999999999999</v>
+        <v>75.5</v>
       </c>
       <c r="M53" t="n">
         <v>4.509</v>
       </c>
       <c r="N53" t="n">
-        <v>85.40000000000001</v>
+        <v>81.3</v>
       </c>
       <c r="O53" t="inlineStr"/>
       <c r="P53" t="inlineStr">
@@ -3195,13 +3195,13 @@
         <v>3.872</v>
       </c>
       <c r="L54" t="n">
-        <v>12.3</v>
+        <v>12.5</v>
       </c>
       <c r="M54" t="n">
         <v>3.88</v>
       </c>
       <c r="N54" t="n">
-        <v>18.9</v>
+        <v>18.2</v>
       </c>
       <c r="O54" t="inlineStr"/>
       <c r="P54" t="inlineStr">
@@ -3247,13 +3247,13 @@
         <v>3.937</v>
       </c>
       <c r="L55" t="n">
-        <v>17.6</v>
+        <v>18</v>
       </c>
       <c r="M55" t="n">
         <v>3.866</v>
       </c>
       <c r="N55" t="n">
-        <v>16.8</v>
+        <v>16.2</v>
       </c>
       <c r="O55" t="inlineStr"/>
       <c r="P55" t="inlineStr">
@@ -3299,13 +3299,13 @@
         <v>4.29</v>
       </c>
       <c r="L56" t="n">
-        <v>67.40000000000001</v>
+        <v>65.5</v>
       </c>
       <c r="M56" t="n">
         <v>4.415</v>
       </c>
       <c r="N56" t="n">
-        <v>74.59999999999999</v>
+        <v>71.2</v>
       </c>
       <c r="O56" t="inlineStr"/>
       <c r="P56" t="inlineStr">
@@ -3351,13 +3351,13 @@
         <v>4.143</v>
       </c>
       <c r="L57" t="n">
-        <v>40.1</v>
+        <v>39</v>
       </c>
       <c r="M57" t="n">
         <v>4.068</v>
       </c>
       <c r="N57" t="n">
-        <v>31.9</v>
+        <v>30.3</v>
       </c>
       <c r="O57" t="inlineStr"/>
       <c r="P57" t="inlineStr">
@@ -3399,13 +3399,13 @@
         <v>4.316</v>
       </c>
       <c r="L58" t="n">
-        <v>73.8</v>
+        <v>71.5</v>
       </c>
       <c r="M58" t="n">
         <v>4.442</v>
       </c>
       <c r="N58" t="n">
-        <v>76.8</v>
+        <v>73.2</v>
       </c>
       <c r="O58" t="inlineStr"/>
       <c r="P58" t="inlineStr">
@@ -3451,13 +3451,13 @@
         <v>3.801</v>
       </c>
       <c r="L59" t="n">
-        <v>4.3</v>
+        <v>5</v>
       </c>
       <c r="M59" t="n">
         <v>3.555</v>
       </c>
       <c r="N59" t="n">
-        <v>4.9</v>
+        <v>4.5</v>
       </c>
       <c r="O59" t="inlineStr"/>
       <c r="P59" t="inlineStr">
@@ -3503,13 +3503,13 @@
         <v>4.424</v>
       </c>
       <c r="L60" t="n">
-        <v>88.8</v>
+        <v>87</v>
       </c>
       <c r="M60" t="n">
         <v>4.553</v>
       </c>
       <c r="N60" t="n">
-        <v>89.2</v>
+        <v>84.8</v>
       </c>
       <c r="O60" t="inlineStr"/>
       <c r="P60" t="inlineStr">
@@ -3555,13 +3555,13 @@
         <v>4.647</v>
       </c>
       <c r="L61" t="n">
-        <v>98.40000000000001</v>
+        <v>97.5</v>
       </c>
       <c r="M61" t="n">
         <v>4.611</v>
       </c>
       <c r="N61" t="n">
-        <v>94.09999999999999</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="O61" t="inlineStr"/>
       <c r="P61" t="inlineStr">
@@ -3607,13 +3607,13 @@
         <v>3.782</v>
       </c>
       <c r="L62" t="n">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="M62" t="n">
         <v>3.73</v>
       </c>
       <c r="N62" t="n">
-        <v>9.699999999999999</v>
+        <v>9.6</v>
       </c>
       <c r="O62" t="inlineStr"/>
       <c r="P62" t="inlineStr">
@@ -3659,13 +3659,13 @@
         <v>4.138</v>
       </c>
       <c r="L63" t="n">
-        <v>37.4</v>
+        <v>36.5</v>
       </c>
       <c r="M63" t="n">
         <v>3.913</v>
       </c>
       <c r="N63" t="n">
-        <v>22.7</v>
+        <v>21.7</v>
       </c>
       <c r="O63" t="inlineStr"/>
       <c r="P63" t="inlineStr">
@@ -3711,13 +3711,13 @@
         <v>4.084</v>
       </c>
       <c r="L64" t="n">
-        <v>29.9</v>
+        <v>29.5</v>
       </c>
       <c r="M64" t="n">
         <v>4.377</v>
       </c>
       <c r="N64" t="n">
-        <v>67.59999999999999</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="O64" t="inlineStr"/>
       <c r="P64" t="inlineStr">
@@ -3759,13 +3759,13 @@
         <v>4.397</v>
       </c>
       <c r="L65" t="n">
-        <v>86.09999999999999</v>
+        <v>84</v>
       </c>
       <c r="M65" t="n">
         <v>4.359</v>
       </c>
       <c r="N65" t="n">
-        <v>65.90000000000001</v>
+        <v>63.1</v>
       </c>
       <c r="O65" t="inlineStr"/>
       <c r="P65" t="inlineStr">
@@ -3811,13 +3811,13 @@
         <v>4.067</v>
       </c>
       <c r="L66" t="n">
-        <v>27.8</v>
+        <v>27.5</v>
       </c>
       <c r="M66" t="n">
         <v>4.186</v>
       </c>
       <c r="N66" t="n">
-        <v>43.8</v>
+        <v>41.9</v>
       </c>
       <c r="O66" t="inlineStr"/>
       <c r="P66" t="inlineStr">
@@ -3863,13 +3863,13 @@
         <v>4.168</v>
       </c>
       <c r="L67" t="n">
-        <v>43.3</v>
+        <v>42</v>
       </c>
       <c r="M67" t="n">
         <v>4.189</v>
       </c>
       <c r="N67" t="n">
-        <v>44.9</v>
+        <v>42.9</v>
       </c>
       <c r="O67" t="inlineStr"/>
       <c r="P67" t="inlineStr">
@@ -3915,13 +3915,13 @@
         <v>4.328</v>
       </c>
       <c r="L68" t="n">
-        <v>75.90000000000001</v>
+        <v>73.5</v>
       </c>
       <c r="M68" t="n">
         <v>4.498</v>
       </c>
       <c r="N68" t="n">
-        <v>84.3</v>
+        <v>80.3</v>
       </c>
       <c r="O68" t="inlineStr"/>
       <c r="P68" t="inlineStr">
@@ -3963,13 +3963,13 @@
         <v>4.25</v>
       </c>
       <c r="L69" t="n">
-        <v>53.5</v>
+        <v>52</v>
       </c>
       <c r="M69" t="n">
         <v>4.272</v>
       </c>
       <c r="N69" t="n">
-        <v>55.7</v>
+        <v>53.5</v>
       </c>
       <c r="O69" t="inlineStr"/>
       <c r="P69" t="inlineStr">
@@ -4011,13 +4011,13 @@
         <v>4.222</v>
       </c>
       <c r="L70" t="n">
-        <v>49.7</v>
+        <v>48.5</v>
       </c>
       <c r="M70" t="n">
         <v>4.375</v>
       </c>
       <c r="N70" t="n">
-        <v>67</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="O70" t="inlineStr"/>
       <c r="P70" t="inlineStr">
@@ -4063,13 +4063,13 @@
         <v>4.403</v>
       </c>
       <c r="L71" t="n">
-        <v>87.2</v>
+        <v>85</v>
       </c>
       <c r="M71" t="n">
         <v>4.412</v>
       </c>
       <c r="N71" t="n">
-        <v>74.09999999999999</v>
+        <v>70.7</v>
       </c>
       <c r="O71" t="inlineStr"/>
       <c r="P71" t="inlineStr">
@@ -4115,13 +4115,13 @@
         <v>4.229</v>
       </c>
       <c r="L72" t="n">
-        <v>50.8</v>
+        <v>49.5</v>
       </c>
       <c r="M72" t="n">
         <v>4.035</v>
       </c>
       <c r="N72" t="n">
-        <v>29.2</v>
+        <v>27.8</v>
       </c>
       <c r="O72" t="inlineStr"/>
       <c r="P72" t="inlineStr">
@@ -4167,13 +4167,13 @@
         <v>3.884</v>
       </c>
       <c r="L73" t="n">
-        <v>12.8</v>
+        <v>13</v>
       </c>
       <c r="M73" t="n">
         <v>4.101</v>
       </c>
       <c r="N73" t="n">
-        <v>35.1</v>
+        <v>33.3</v>
       </c>
       <c r="O73" t="inlineStr"/>
       <c r="P73" t="inlineStr">
@@ -4219,13 +4219,13 @@
         <v>4.309</v>
       </c>
       <c r="L74" t="n">
-        <v>71.7</v>
+        <v>69.5</v>
       </c>
       <c r="M74" t="n">
         <v>4.313</v>
       </c>
       <c r="N74" t="n">
-        <v>61.1</v>
+        <v>58.6</v>
       </c>
       <c r="O74" t="inlineStr"/>
       <c r="P74" t="inlineStr">
@@ -4271,13 +4271,13 @@
         <v>4.357</v>
       </c>
       <c r="L75" t="n">
-        <v>80.7</v>
+        <v>78</v>
       </c>
       <c r="M75" t="n">
         <v>4.408</v>
       </c>
       <c r="N75" t="n">
-        <v>73</v>
+        <v>69.7</v>
       </c>
       <c r="O75" t="inlineStr"/>
       <c r="P75" t="inlineStr">
@@ -4319,13 +4319,13 @@
         <v>4.114</v>
       </c>
       <c r="L76" t="n">
-        <v>34.2</v>
+        <v>33.5</v>
       </c>
       <c r="M76" t="n">
         <v>4.217</v>
       </c>
       <c r="N76" t="n">
-        <v>49.2</v>
+        <v>47.5</v>
       </c>
       <c r="O76" t="inlineStr"/>
       <c r="P76" t="inlineStr">
@@ -4371,13 +4371,13 @@
         <v>4.14</v>
       </c>
       <c r="L77" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="M77" t="n">
         <v>3.525</v>
       </c>
       <c r="N77" t="n">
-        <v>2.7</v>
+        <v>2.5</v>
       </c>
       <c r="O77" t="inlineStr"/>
       <c r="P77" t="inlineStr">
@@ -4419,13 +4419,13 @@
         <v>4.454</v>
       </c>
       <c r="L78" t="n">
-        <v>91.40000000000001</v>
+        <v>90</v>
       </c>
       <c r="M78" t="n">
         <v>4.506</v>
       </c>
       <c r="N78" t="n">
-        <v>84.90000000000001</v>
+        <v>80.8</v>
       </c>
       <c r="O78" t="inlineStr"/>
       <c r="P78" t="inlineStr">
@@ -4471,13 +4471,13 @@
         <v>4.277</v>
       </c>
       <c r="L79" t="n">
-        <v>62.6</v>
+        <v>60.5</v>
       </c>
       <c r="M79" t="n">
         <v>4.299</v>
       </c>
       <c r="N79" t="n">
-        <v>58.9</v>
+        <v>56.6</v>
       </c>
       <c r="O79" t="inlineStr"/>
       <c r="P79" t="inlineStr">
@@ -4523,13 +4523,13 @@
         <v>4.188</v>
       </c>
       <c r="L80" t="n">
-        <v>45.5</v>
+        <v>44.5</v>
       </c>
       <c r="M80" t="n">
         <v>4.022</v>
       </c>
       <c r="N80" t="n">
-        <v>28.1</v>
+        <v>26.8</v>
       </c>
       <c r="O80" t="inlineStr"/>
       <c r="P80" t="inlineStr">
@@ -4575,13 +4575,13 @@
         <v>4.021</v>
       </c>
       <c r="L81" t="n">
-        <v>25.7</v>
+        <v>25.5</v>
       </c>
       <c r="M81" t="n">
         <v>4.064</v>
       </c>
       <c r="N81" t="n">
-        <v>31.4</v>
+        <v>29.8</v>
       </c>
       <c r="O81" t="inlineStr"/>
       <c r="P81" t="inlineStr">
@@ -4627,13 +4627,13 @@
         <v>4.352</v>
       </c>
       <c r="L82" t="n">
-        <v>79.09999999999999</v>
+        <v>76.5</v>
       </c>
       <c r="M82" t="n">
         <v>4.223</v>
       </c>
       <c r="N82" t="n">
-        <v>50.3</v>
+        <v>48.5</v>
       </c>
       <c r="O82" t="inlineStr"/>
       <c r="P82" t="inlineStr">
@@ -4679,13 +4679,13 @@
         <v>4.156</v>
       </c>
       <c r="L83" t="n">
-        <v>42.2</v>
+        <v>41</v>
       </c>
       <c r="M83" t="n">
         <v>3.991</v>
       </c>
       <c r="N83" t="n">
-        <v>26.5</v>
+        <v>25.3</v>
       </c>
       <c r="O83" t="inlineStr"/>
       <c r="P83" t="inlineStr">
@@ -4737,7 +4737,7 @@
         <v>4.488</v>
       </c>
       <c r="N84" t="n">
-        <v>83.2</v>
+        <v>79.3</v>
       </c>
       <c r="O84" t="inlineStr"/>
       <c r="P84" t="inlineStr">
@@ -4783,13 +4783,13 @@
         <v>4.289</v>
       </c>
       <c r="L85" t="n">
-        <v>66.8</v>
+        <v>64.5</v>
       </c>
       <c r="M85" t="n">
         <v>4.256</v>
       </c>
       <c r="N85" t="n">
-        <v>54.1</v>
+        <v>52</v>
       </c>
       <c r="O85" t="inlineStr"/>
       <c r="P85" t="inlineStr">
@@ -4835,13 +4835,13 @@
         <v>4.197</v>
       </c>
       <c r="L86" s="2" t="n">
-        <v>46.5</v>
+        <v>45.5</v>
       </c>
       <c r="M86" s="2" t="n">
         <v>4.382</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>68.59999999999999</v>
+        <v>65.7</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -4891,13 +4891,13 @@
         <v>4.353</v>
       </c>
       <c r="L87" t="n">
-        <v>79.7</v>
+        <v>77</v>
       </c>
       <c r="M87" t="n">
         <v>4.48</v>
       </c>
       <c r="N87" t="n">
-        <v>82.2</v>
+        <v>78.3</v>
       </c>
       <c r="O87" t="inlineStr"/>
       <c r="P87" t="inlineStr">
@@ -4943,13 +4943,13 @@
         <v>4.298</v>
       </c>
       <c r="L88" t="n">
-        <v>70.09999999999999</v>
+        <v>68</v>
       </c>
       <c r="M88" t="n">
         <v>4.127</v>
       </c>
       <c r="N88" t="n">
-        <v>37.3</v>
+        <v>35.4</v>
       </c>
       <c r="O88" t="inlineStr"/>
       <c r="P88" t="inlineStr">
@@ -4995,13 +4995,13 @@
         <v>4.207</v>
       </c>
       <c r="L89" t="n">
-        <v>47.6</v>
+        <v>46.5</v>
       </c>
       <c r="M89" t="n">
         <v>4.252</v>
       </c>
       <c r="N89" t="n">
-        <v>53.5</v>
+        <v>51.5</v>
       </c>
       <c r="O89" t="inlineStr"/>
       <c r="P89" t="inlineStr">
@@ -5047,13 +5047,13 @@
         <v>4.519</v>
       </c>
       <c r="L90" t="n">
-        <v>95.2</v>
+        <v>94.5</v>
       </c>
       <c r="M90" t="n">
         <v>4.405</v>
       </c>
       <c r="N90" t="n">
-        <v>71.40000000000001</v>
+        <v>68.2</v>
       </c>
       <c r="O90" t="inlineStr"/>
       <c r="P90" t="inlineStr">
@@ -5099,13 +5099,13 @@
         <v>4.335</v>
       </c>
       <c r="L91" t="n">
-        <v>77</v>
+        <v>74.5</v>
       </c>
       <c r="M91" t="n">
         <v>4.406</v>
       </c>
       <c r="N91" t="n">
-        <v>71.90000000000001</v>
+        <v>68.7</v>
       </c>
       <c r="O91" t="inlineStr"/>
       <c r="P91" t="inlineStr">
@@ -5151,13 +5151,13 @@
         <v>3.892</v>
       </c>
       <c r="L92" t="n">
-        <v>13.9</v>
+        <v>14</v>
       </c>
       <c r="M92" t="n">
         <v>3.933</v>
       </c>
       <c r="N92" t="n">
-        <v>23.2</v>
+        <v>22.2</v>
       </c>
       <c r="O92" t="inlineStr"/>
       <c r="P92" t="inlineStr">
@@ -5203,13 +5203,13 @@
         <v>4.297</v>
       </c>
       <c r="L93" t="n">
-        <v>69.5</v>
+        <v>67.5</v>
       </c>
       <c r="M93" t="n">
         <v>4.605</v>
       </c>
       <c r="N93" t="n">
-        <v>91.90000000000001</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="O93" t="inlineStr"/>
       <c r="P93" t="inlineStr">
@@ -5255,13 +5255,13 @@
         <v>4.291</v>
       </c>
       <c r="L94" t="n">
-        <v>67.90000000000001</v>
+        <v>66</v>
       </c>
       <c r="M94" t="n">
         <v>4.134</v>
       </c>
       <c r="N94" t="n">
-        <v>38.9</v>
+        <v>36.9</v>
       </c>
       <c r="O94" t="inlineStr"/>
       <c r="P94" t="inlineStr">
@@ -5307,13 +5307,13 @@
         <v>4.324</v>
       </c>
       <c r="L95" t="n">
-        <v>74.90000000000001</v>
+        <v>72.5</v>
       </c>
       <c r="M95" t="n">
         <v>4.264</v>
       </c>
       <c r="N95" t="n">
-        <v>54.6</v>
+        <v>52.5</v>
       </c>
       <c r="O95" t="inlineStr"/>
       <c r="P95" t="inlineStr">
@@ -5359,13 +5359,13 @@
         <v>4.72</v>
       </c>
       <c r="L96" t="n">
-        <v>98.90000000000001</v>
+        <v>99</v>
       </c>
       <c r="M96" t="n">
         <v>4.679</v>
       </c>
       <c r="N96" t="n">
-        <v>96.8</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="O96" t="inlineStr"/>
       <c r="P96" t="inlineStr">
@@ -5411,13 +5411,13 @@
         <v>4.37</v>
       </c>
       <c r="L97" t="n">
-        <v>82.90000000000001</v>
+        <v>80.5</v>
       </c>
       <c r="M97" t="n">
         <v>4.416</v>
       </c>
       <c r="N97" t="n">
-        <v>75.09999999999999</v>
+        <v>71.7</v>
       </c>
       <c r="O97" t="inlineStr"/>
       <c r="P97" t="inlineStr">
@@ -5459,13 +5459,13 @@
         <v>4.266</v>
       </c>
       <c r="L98" t="n">
-        <v>59.9</v>
+        <v>58</v>
       </c>
       <c r="M98" t="n">
         <v>4.391</v>
       </c>
       <c r="N98" t="n">
-        <v>69.7</v>
+        <v>66.7</v>
       </c>
       <c r="O98" t="inlineStr"/>
       <c r="P98" t="inlineStr">
@@ -5507,13 +5507,13 @@
         <v>4.069</v>
       </c>
       <c r="L99" t="n">
-        <v>28.3</v>
+        <v>28</v>
       </c>
       <c r="M99" t="n">
         <v>4.09</v>
       </c>
       <c r="N99" t="n">
-        <v>34.1</v>
+        <v>32.3</v>
       </c>
       <c r="O99" t="inlineStr"/>
       <c r="P99" t="inlineStr">
@@ -5555,13 +5555,13 @@
         <v>4.299</v>
       </c>
       <c r="L100" t="n">
-        <v>70.59999999999999</v>
+        <v>68.5</v>
       </c>
       <c r="M100" t="n">
         <v>4.462</v>
       </c>
       <c r="N100" t="n">
-        <v>80</v>
+        <v>76.3</v>
       </c>
       <c r="O100" t="inlineStr"/>
       <c r="P100" t="inlineStr">
@@ -5603,13 +5603,13 @@
         <v>4.383</v>
       </c>
       <c r="L101" t="n">
-        <v>84</v>
+        <v>81.5</v>
       </c>
       <c r="M101" t="n">
         <v>4.555</v>
       </c>
       <c r="N101" t="n">
-        <v>89.7</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="O101" t="inlineStr"/>
       <c r="P101" t="inlineStr">
@@ -5657,7 +5657,7 @@
         <v>3.846</v>
       </c>
       <c r="N102" t="n">
-        <v>15.1</v>
+        <v>14.6</v>
       </c>
       <c r="O102" t="inlineStr"/>
       <c r="P102" t="inlineStr">
@@ -5699,13 +5699,13 @@
         <v>4.313</v>
       </c>
       <c r="L103" t="n">
-        <v>72.7</v>
+        <v>70.5</v>
       </c>
       <c r="M103" t="n">
         <v>4.579</v>
       </c>
       <c r="N103" t="n">
-        <v>90.8</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="O103" t="inlineStr"/>
       <c r="P103" t="inlineStr">
@@ -5751,13 +5751,13 @@
         <v>4.14</v>
       </c>
       <c r="L104" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="M104" t="n">
         <v>4.049</v>
       </c>
       <c r="N104" t="n">
-        <v>30.3</v>
+        <v>28.8</v>
       </c>
       <c r="O104" t="inlineStr"/>
       <c r="P104" t="inlineStr">
@@ -5803,13 +5803,13 @@
         <v>4.032</v>
       </c>
       <c r="L105" t="n">
-        <v>26.2</v>
+        <v>26</v>
       </c>
       <c r="M105" t="n">
         <v>3.872</v>
       </c>
       <c r="N105" t="n">
-        <v>17.8</v>
+        <v>17.2</v>
       </c>
       <c r="O105" t="inlineStr"/>
       <c r="P105" t="inlineStr">
@@ -5847,13 +5847,13 @@
         <v>4.228</v>
       </c>
       <c r="L106" t="n">
-        <v>50.3</v>
+        <v>49</v>
       </c>
       <c r="M106" t="n">
         <v>4.282</v>
       </c>
       <c r="N106" t="n">
-        <v>58.4</v>
+        <v>56.1</v>
       </c>
       <c r="O106" t="inlineStr"/>
       <c r="P106" t="inlineStr">
@@ -5899,13 +5899,13 @@
         <v>4.614</v>
       </c>
       <c r="L107" t="n">
-        <v>97.3</v>
+        <v>96.5</v>
       </c>
       <c r="M107" t="n">
         <v>4.531</v>
       </c>
       <c r="N107" t="n">
-        <v>87</v>
+        <v>82.8</v>
       </c>
       <c r="O107" t="inlineStr"/>
       <c r="P107" t="inlineStr">
@@ -5947,13 +5947,13 @@
         <v>4.201</v>
       </c>
       <c r="L108" t="n">
-        <v>47.1</v>
+        <v>46</v>
       </c>
       <c r="M108" t="n">
         <v>4.421</v>
       </c>
       <c r="N108" t="n">
-        <v>75.7</v>
+        <v>72.2</v>
       </c>
       <c r="O108" t="inlineStr"/>
       <c r="P108" t="inlineStr">
@@ -5995,13 +5995,13 @@
         <v>4.211</v>
       </c>
       <c r="L109" t="n">
-        <v>48.1</v>
+        <v>47</v>
       </c>
       <c r="M109" t="n">
         <v>4.22</v>
       </c>
       <c r="N109" t="n">
-        <v>49.7</v>
+        <v>48</v>
       </c>
       <c r="O109" t="inlineStr"/>
       <c r="P109" t="inlineStr">
@@ -6043,13 +6043,13 @@
         <v>3.87</v>
       </c>
       <c r="L110" t="n">
-        <v>10.7</v>
+        <v>11</v>
       </c>
       <c r="M110" t="n">
         <v>3.878</v>
       </c>
       <c r="N110" t="n">
-        <v>18.4</v>
+        <v>17.7</v>
       </c>
       <c r="O110" t="inlineStr"/>
       <c r="P110" t="inlineStr">
@@ -6091,13 +6091,13 @@
         <v>3.871</v>
       </c>
       <c r="L111" t="n">
-        <v>11.2</v>
+        <v>11.5</v>
       </c>
       <c r="M111" t="n">
         <v>4.074</v>
       </c>
       <c r="N111" t="n">
-        <v>32.4</v>
+        <v>30.8</v>
       </c>
       <c r="O111" t="inlineStr"/>
       <c r="P111" t="inlineStr">
@@ -6135,13 +6135,13 @@
         <v>4.264</v>
       </c>
       <c r="L112" t="n">
-        <v>57.2</v>
+        <v>55.5</v>
       </c>
       <c r="M112" t="n">
         <v>4.432</v>
       </c>
       <c r="N112" t="n">
-        <v>76.2</v>
+        <v>72.7</v>
       </c>
       <c r="O112" t="inlineStr"/>
       <c r="P112" t="inlineStr">
@@ -6187,13 +6187,13 @@
         <v>4.457</v>
       </c>
       <c r="L113" t="n">
-        <v>92</v>
+        <v>90.5</v>
       </c>
       <c r="M113" t="n">
         <v>4.587</v>
       </c>
       <c r="N113" t="n">
-        <v>91.40000000000001</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="O113" t="inlineStr"/>
       <c r="P113" t="inlineStr">
@@ -6239,13 +6239,13 @@
         <v>4.265</v>
       </c>
       <c r="L114" t="n">
-        <v>59.4</v>
+        <v>57.5</v>
       </c>
       <c r="M114" t="n">
         <v>4.335</v>
       </c>
       <c r="N114" t="n">
-        <v>63.2</v>
+        <v>60.6</v>
       </c>
       <c r="O114" t="inlineStr"/>
       <c r="P114" t="inlineStr">
@@ -6291,13 +6291,13 @@
         <v>4.492</v>
       </c>
       <c r="L115" t="n">
-        <v>94.09999999999999</v>
+        <v>93.5</v>
       </c>
       <c r="M115" t="n">
         <v>4.411</v>
       </c>
       <c r="N115" t="n">
-        <v>73.5</v>
+        <v>70.2</v>
       </c>
       <c r="O115" t="inlineStr"/>
       <c r="P115" t="inlineStr">
@@ -6335,13 +6335,13 @@
         <v>4.401</v>
       </c>
       <c r="L116" t="n">
-        <v>86.59999999999999</v>
+        <v>84.5</v>
       </c>
       <c r="M116" t="n">
         <v>4.473</v>
       </c>
       <c r="N116" t="n">
-        <v>81.09999999999999</v>
+        <v>77.3</v>
       </c>
       <c r="O116" t="inlineStr"/>
       <c r="P116" t="inlineStr">
@@ -6387,13 +6387,13 @@
         <v>4.264</v>
       </c>
       <c r="L117" t="n">
-        <v>57.2</v>
+        <v>55.5</v>
       </c>
       <c r="M117" t="n">
         <v>4.17</v>
       </c>
       <c r="N117" t="n">
-        <v>42.7</v>
+        <v>40.9</v>
       </c>
       <c r="O117" t="inlineStr"/>
       <c r="P117" t="inlineStr">
@@ -6435,13 +6435,13 @@
         <v>4.277</v>
       </c>
       <c r="L118" t="n">
-        <v>62.6</v>
+        <v>60.5</v>
       </c>
       <c r="M118" t="n">
         <v>4.2</v>
       </c>
       <c r="N118" t="n">
-        <v>46.5</v>
+        <v>44.4</v>
       </c>
       <c r="O118" t="inlineStr"/>
       <c r="P118" t="inlineStr">
@@ -6483,13 +6483,13 @@
         <v>4.262</v>
       </c>
       <c r="L119" t="n">
-        <v>56.7</v>
+        <v>55</v>
       </c>
       <c r="M119" t="n">
         <v>4.312</v>
       </c>
       <c r="N119" t="n">
-        <v>60.5</v>
+        <v>58.1</v>
       </c>
       <c r="O119" t="inlineStr"/>
       <c r="P119" t="inlineStr">
@@ -6535,13 +6535,13 @@
         <v>3.885</v>
       </c>
       <c r="L120" t="n">
-        <v>13.4</v>
+        <v>13.5</v>
       </c>
       <c r="M120" t="n">
         <v>4.089</v>
       </c>
       <c r="N120" t="n">
-        <v>33.5</v>
+        <v>31.8</v>
       </c>
       <c r="O120" t="inlineStr"/>
       <c r="P120" t="inlineStr">
@@ -6583,13 +6583,13 @@
         <v>4.367</v>
       </c>
       <c r="L121" t="n">
-        <v>81.8</v>
+        <v>79</v>
       </c>
       <c r="M121" t="n">
         <v>4.545</v>
       </c>
       <c r="N121" t="n">
-        <v>88.59999999999999</v>
+        <v>84.3</v>
       </c>
       <c r="O121" t="inlineStr"/>
       <c r="P121" t="inlineStr">
@@ -6631,13 +6631,13 @@
         <v>3.867</v>
       </c>
       <c r="L122" t="n">
-        <v>9.6</v>
+        <v>10</v>
       </c>
       <c r="M122" t="n">
         <v>3.782</v>
       </c>
       <c r="N122" t="n">
-        <v>11.4</v>
+        <v>11.1</v>
       </c>
       <c r="O122" t="inlineStr"/>
       <c r="P122" t="inlineStr">
@@ -6683,13 +6683,13 @@
         <v>4.135</v>
       </c>
       <c r="L123" t="n">
-        <v>36.4</v>
+        <v>35.5</v>
       </c>
       <c r="M123" t="n">
         <v>4.156</v>
       </c>
       <c r="N123" t="n">
-        <v>41.1</v>
+        <v>38.9</v>
       </c>
       <c r="O123" t="inlineStr"/>
       <c r="P123" t="inlineStr">
@@ -6727,13 +6727,13 @@
         <v>4.143</v>
       </c>
       <c r="L124" t="n">
-        <v>40.1</v>
+        <v>39</v>
       </c>
       <c r="M124" t="n">
         <v>4.192</v>
       </c>
       <c r="N124" t="n">
-        <v>45.9</v>
+        <v>43.9</v>
       </c>
       <c r="O124" t="inlineStr"/>
       <c r="P124" t="inlineStr">
@@ -6771,13 +6771,13 @@
         <v>4.115</v>
       </c>
       <c r="L125" t="n">
-        <v>35.3</v>
+        <v>34.5</v>
       </c>
       <c r="M125" t="n">
         <v>4.235</v>
       </c>
       <c r="N125" t="n">
-        <v>51.4</v>
+        <v>49.5</v>
       </c>
       <c r="O125" t="inlineStr"/>
       <c r="P125" t="inlineStr">
@@ -6823,13 +6823,13 @@
         <v>4.26</v>
       </c>
       <c r="L126" t="n">
-        <v>55.6</v>
+        <v>54</v>
       </c>
       <c r="M126" t="n">
         <v>4.448</v>
       </c>
       <c r="N126" t="n">
-        <v>77.8</v>
+        <v>74.2</v>
       </c>
       <c r="O126" t="inlineStr"/>
       <c r="P126" t="inlineStr">
@@ -6871,13 +6871,13 @@
         <v>4.349</v>
       </c>
       <c r="L127" t="n">
-        <v>78.59999999999999</v>
+        <v>76</v>
       </c>
       <c r="M127" t="n">
         <v>4.278</v>
       </c>
       <c r="N127" t="n">
-        <v>57.3</v>
+        <v>55.1</v>
       </c>
       <c r="O127" t="inlineStr"/>
       <c r="P127" t="inlineStr">
@@ -6915,13 +6915,13 @@
         <v>4.095</v>
       </c>
       <c r="L128" t="n">
-        <v>31</v>
+        <v>30.5</v>
       </c>
       <c r="M128" t="n">
         <v>4.021</v>
       </c>
       <c r="N128" t="n">
-        <v>27.6</v>
+        <v>26.3</v>
       </c>
       <c r="O128" t="inlineStr"/>
       <c r="P128" t="inlineStr">
@@ -6967,13 +6967,13 @@
         <v>4.053</v>
       </c>
       <c r="L129" t="n">
-        <v>27.3</v>
+        <v>27</v>
       </c>
       <c r="M129" t="n">
         <v>4.16</v>
       </c>
       <c r="N129" t="n">
-        <v>41.6</v>
+        <v>39.4</v>
       </c>
       <c r="O129" t="inlineStr"/>
       <c r="P129" t="inlineStr">
@@ -7011,13 +7011,13 @@
         <v>3.697</v>
       </c>
       <c r="L130" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="M130" t="n">
         <v>3.805</v>
       </c>
       <c r="N130" t="n">
-        <v>11.9</v>
+        <v>11.6</v>
       </c>
       <c r="O130" t="inlineStr"/>
       <c r="P130" t="inlineStr">
@@ -7055,13 +7055,13 @@
         <v>3.82</v>
       </c>
       <c r="L131" t="n">
-        <v>5.3</v>
+        <v>6</v>
       </c>
       <c r="M131" t="n">
         <v>3.869</v>
       </c>
       <c r="N131" t="n">
-        <v>17.3</v>
+        <v>16.7</v>
       </c>
       <c r="O131" t="inlineStr"/>
       <c r="P131" t="inlineStr">
@@ -7103,13 +7103,13 @@
         <v>3.864</v>
       </c>
       <c r="L132" t="n">
-        <v>7</v>
+        <v>7.5</v>
       </c>
       <c r="M132" t="n">
         <v>4.33</v>
       </c>
       <c r="N132" t="n">
-        <v>62.2</v>
+        <v>59.6</v>
       </c>
       <c r="O132" t="inlineStr"/>
       <c r="P132" t="inlineStr">
@@ -7155,13 +7155,13 @@
         <v>4.178</v>
       </c>
       <c r="L133" t="n">
-        <v>44.4</v>
+        <v>43</v>
       </c>
       <c r="M133" t="n">
         <v>4.336</v>
       </c>
       <c r="N133" t="n">
-        <v>63.8</v>
+        <v>61.1</v>
       </c>
       <c r="O133" t="inlineStr"/>
       <c r="P133" t="inlineStr">
@@ -7207,13 +7207,13 @@
         <v>4.386</v>
       </c>
       <c r="L134" t="n">
-        <v>84.5</v>
+        <v>82</v>
       </c>
       <c r="M134" t="n">
         <v>4.656</v>
       </c>
       <c r="N134" t="n">
-        <v>96.2</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="O134" t="inlineStr"/>
       <c r="P134" t="inlineStr">
@@ -7259,13 +7259,13 @@
         <v>3.906</v>
       </c>
       <c r="L135" t="n">
-        <v>15</v>
+        <v>15.5</v>
       </c>
       <c r="M135" t="n">
         <v>4.281</v>
       </c>
       <c r="N135" t="n">
-        <v>57.8</v>
+        <v>55.6</v>
       </c>
       <c r="O135" t="inlineStr"/>
       <c r="P135" t="inlineStr">
@@ -7311,13 +7311,13 @@
         <v>4.136</v>
       </c>
       <c r="L136" t="n">
-        <v>36.9</v>
+        <v>36</v>
       </c>
       <c r="M136" t="n">
         <v>3.985</v>
       </c>
       <c r="N136" t="n">
-        <v>25.9</v>
+        <v>24.7</v>
       </c>
       <c r="O136" t="inlineStr"/>
       <c r="P136" t="inlineStr">
@@ -7363,13 +7363,13 @@
         <v>4.479</v>
       </c>
       <c r="L137" t="n">
-        <v>93.59999999999999</v>
+        <v>92</v>
       </c>
       <c r="M137" t="n">
         <v>4.61</v>
       </c>
       <c r="N137" t="n">
-        <v>93.5</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="O137" t="inlineStr"/>
       <c r="P137" t="inlineStr">
@@ -7415,13 +7415,13 @@
         <v>3.783</v>
       </c>
       <c r="L138" t="n">
-        <v>3.7</v>
+        <v>4.5</v>
       </c>
       <c r="M138" t="n">
         <v>3.362</v>
       </c>
       <c r="N138" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="O138" t="inlineStr"/>
       <c r="P138" t="inlineStr">
@@ -7467,13 +7467,13 @@
         <v>4.438</v>
       </c>
       <c r="L139" t="n">
-        <v>89.8</v>
+        <v>88.5</v>
       </c>
       <c r="M139" t="n">
         <v>4.365</v>
       </c>
       <c r="N139" t="n">
-        <v>66.5</v>
+        <v>63.6</v>
       </c>
       <c r="O139" t="inlineStr"/>
       <c r="P139" t="inlineStr">
@@ -7511,13 +7511,13 @@
         <v>4.271</v>
       </c>
       <c r="L140" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="M140" t="n">
         <v>4.101</v>
       </c>
       <c r="N140" t="n">
-        <v>35.1</v>
+        <v>33.3</v>
       </c>
       <c r="O140" t="inlineStr"/>
       <c r="P140" t="inlineStr">
@@ -7563,13 +7563,13 @@
         <v>3.52</v>
       </c>
       <c r="L141" t="n">
-        <v>1.1</v>
+        <v>1.5</v>
       </c>
       <c r="M141" t="n">
         <v>3.599</v>
       </c>
       <c r="N141" t="n">
-        <v>7</v>
+        <v>7.1</v>
       </c>
       <c r="O141" t="inlineStr"/>
       <c r="P141" t="inlineStr">
@@ -7615,13 +7615,13 @@
         <v>4.171</v>
       </c>
       <c r="L142" t="n">
-        <v>43.9</v>
+        <v>42.5</v>
       </c>
       <c r="M142" t="n">
         <v>4.131</v>
       </c>
       <c r="N142" t="n">
-        <v>38.4</v>
+        <v>36.4</v>
       </c>
       <c r="O142" t="inlineStr"/>
       <c r="P142" t="inlineStr">
@@ -7667,13 +7667,13 @@
         <v>4.323</v>
       </c>
       <c r="L143" t="n">
-        <v>74.3</v>
+        <v>72</v>
       </c>
       <c r="M143" t="n">
         <v>4.606</v>
       </c>
       <c r="N143" t="n">
-        <v>92.40000000000001</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="O143" t="inlineStr"/>
       <c r="P143" t="inlineStr">
@@ -7711,13 +7711,13 @@
         <v>4.282</v>
       </c>
       <c r="L144" t="n">
-        <v>64.2</v>
+        <v>62</v>
       </c>
       <c r="M144" t="n">
         <v>4.205</v>
       </c>
       <c r="N144" t="n">
-        <v>47.6</v>
+        <v>46</v>
       </c>
       <c r="O144" t="inlineStr"/>
       <c r="P144" t="inlineStr">
@@ -7763,13 +7763,13 @@
         <v>4.189</v>
       </c>
       <c r="L145" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="M145" t="n">
         <v>4.341</v>
       </c>
       <c r="N145" t="n">
-        <v>64.3</v>
+        <v>61.6</v>
       </c>
       <c r="O145" t="inlineStr"/>
       <c r="P145" t="inlineStr">
@@ -7815,13 +7815,13 @@
         <v>4.478</v>
       </c>
       <c r="L146" t="n">
-        <v>93</v>
+        <v>91.5</v>
       </c>
       <c r="M146" t="n">
         <v>4.483</v>
       </c>
       <c r="N146" t="n">
-        <v>82.7</v>
+        <v>78.8</v>
       </c>
       <c r="O146" t="inlineStr"/>
       <c r="P146" t="inlineStr">
@@ -7863,13 +7863,13 @@
         <v>4.42</v>
       </c>
       <c r="L147" t="n">
-        <v>88.2</v>
+        <v>86.5</v>
       </c>
       <c r="M147" t="n">
         <v>4.492</v>
       </c>
       <c r="N147" t="n">
-        <v>83.8</v>
+        <v>79.8</v>
       </c>
       <c r="O147" t="inlineStr"/>
       <c r="P147" t="inlineStr">
@@ -7915,13 +7915,13 @@
         <v>4.286</v>
       </c>
       <c r="L148" t="n">
-        <v>65.8</v>
+        <v>63.5</v>
       </c>
       <c r="M148" t="n">
         <v>4.356</v>
       </c>
       <c r="N148" t="n">
-        <v>65.40000000000001</v>
+        <v>62.6</v>
       </c>
       <c r="O148" t="inlineStr"/>
       <c r="P148" t="inlineStr">
@@ -7967,13 +7967,13 @@
         <v>4.103</v>
       </c>
       <c r="L149" t="n">
-        <v>32.1</v>
+        <v>31.5</v>
       </c>
       <c r="M149" t="n">
         <v>4.17</v>
       </c>
       <c r="N149" t="n">
-        <v>42.7</v>
+        <v>40.9</v>
       </c>
       <c r="O149" t="inlineStr"/>
       <c r="P149" t="inlineStr">
@@ -8019,13 +8019,13 @@
         <v>4.276</v>
       </c>
       <c r="L150" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M150" t="n">
         <v>4.268</v>
       </c>
       <c r="N150" t="n">
-        <v>55.1</v>
+        <v>53</v>
       </c>
       <c r="O150" t="inlineStr"/>
       <c r="P150" t="inlineStr">
@@ -8071,13 +8071,13 @@
         <v>4.38</v>
       </c>
       <c r="L151" t="n">
-        <v>83.40000000000001</v>
+        <v>81</v>
       </c>
       <c r="M151" t="n">
         <v>4.452</v>
       </c>
       <c r="N151" t="n">
-        <v>78.40000000000001</v>
+        <v>74.7</v>
       </c>
       <c r="O151" t="inlineStr"/>
       <c r="P151" t="inlineStr">
@@ -8123,13 +8123,13 @@
         <v>3.943</v>
       </c>
       <c r="L152" t="n">
-        <v>18.2</v>
+        <v>18.5</v>
       </c>
       <c r="M152" t="n">
         <v>4.008</v>
       </c>
       <c r="N152" t="n">
-        <v>27</v>
+        <v>25.8</v>
       </c>
       <c r="O152" t="inlineStr"/>
       <c r="P152" t="inlineStr">
@@ -8175,13 +8175,13 @@
         <v>4.441</v>
       </c>
       <c r="L153" t="n">
-        <v>90.40000000000001</v>
+        <v>89</v>
       </c>
       <c r="M153" t="n">
         <v>4.407</v>
       </c>
       <c r="N153" t="n">
-        <v>72.40000000000001</v>
+        <v>69.2</v>
       </c>
       <c r="O153" t="inlineStr"/>
       <c r="P153" t="inlineStr">
@@ -8227,13 +8227,13 @@
         <v>4.446</v>
       </c>
       <c r="L154" t="n">
-        <v>90.90000000000001</v>
+        <v>89.5</v>
       </c>
       <c r="M154" t="n">
         <v>4.455</v>
       </c>
       <c r="N154" t="n">
-        <v>78.90000000000001</v>
+        <v>75.3</v>
       </c>
       <c r="O154" t="inlineStr"/>
       <c r="P154" t="inlineStr">
@@ -8279,13 +8279,13 @@
         <v>4.286</v>
       </c>
       <c r="L155" t="n">
-        <v>65.8</v>
+        <v>63.5</v>
       </c>
       <c r="M155" t="n">
         <v>4.526</v>
       </c>
       <c r="N155" t="n">
-        <v>86.5</v>
+        <v>82.3</v>
       </c>
       <c r="O155" t="inlineStr"/>
       <c r="P155" t="inlineStr">
@@ -8331,13 +8331,13 @@
         <v>4.312</v>
       </c>
       <c r="L156" t="n">
-        <v>72.2</v>
+        <v>70</v>
       </c>
       <c r="M156" t="n">
         <v>3.71</v>
       </c>
       <c r="N156" t="n">
-        <v>9.199999999999999</v>
+        <v>9.1</v>
       </c>
       <c r="O156" t="inlineStr"/>
       <c r="P156" t="inlineStr">
@@ -8389,7 +8389,7 @@
         <v>3.578</v>
       </c>
       <c r="N157" t="n">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="O157" t="inlineStr"/>
       <c r="P157" t="inlineStr">
@@ -8435,13 +8435,13 @@
         <v>4.277</v>
       </c>
       <c r="L158" t="n">
-        <v>62.6</v>
+        <v>60.5</v>
       </c>
       <c r="M158" t="n">
         <v>3.832</v>
       </c>
       <c r="N158" t="n">
-        <v>14.1</v>
+        <v>13.6</v>
       </c>
       <c r="O158" t="inlineStr"/>
       <c r="P158" t="inlineStr">
@@ -8487,13 +8487,13 @@
         <v>4.109</v>
       </c>
       <c r="L159" t="n">
-        <v>33.2</v>
+        <v>32.5</v>
       </c>
       <c r="M159" t="n">
         <v>3.946</v>
       </c>
       <c r="N159" t="n">
-        <v>23.8</v>
+        <v>22.7</v>
       </c>
       <c r="O159" t="inlineStr"/>
       <c r="P159" t="inlineStr">
@@ -8591,13 +8591,13 @@
         <v>4.436</v>
       </c>
       <c r="L161" t="n">
-        <v>89.3</v>
+        <v>88</v>
       </c>
       <c r="M161" t="n">
         <v>3.862</v>
       </c>
       <c r="N161" t="n">
-        <v>15.7</v>
+        <v>15.2</v>
       </c>
       <c r="O161" t="inlineStr"/>
       <c r="P161" t="inlineStr">
@@ -8643,13 +8643,13 @@
         <v>3.866</v>
       </c>
       <c r="L162" t="n">
-        <v>9.1</v>
+        <v>9.5</v>
       </c>
       <c r="M162" t="n">
         <v>3.573</v>
       </c>
       <c r="N162" t="n">
-        <v>5.9</v>
+        <v>6.1</v>
       </c>
       <c r="O162" t="inlineStr"/>
       <c r="P162" t="inlineStr">
@@ -8695,13 +8695,13 @@
         <v>4.178</v>
       </c>
       <c r="L163" t="n">
-        <v>44.4</v>
+        <v>43</v>
       </c>
       <c r="M163" t="n">
         <v>3.908</v>
       </c>
       <c r="N163" t="n">
-        <v>22.2</v>
+        <v>21.2</v>
       </c>
       <c r="O163" t="inlineStr"/>
       <c r="P163" t="inlineStr">
@@ -8747,13 +8747,13 @@
         <v>4.414</v>
       </c>
       <c r="L164" t="n">
-        <v>87.7</v>
+        <v>86</v>
       </c>
       <c r="M164" t="n">
         <v>4.393</v>
       </c>
       <c r="N164" t="n">
-        <v>70.3</v>
+        <v>67.2</v>
       </c>
       <c r="O164" t="inlineStr"/>
       <c r="P164" t="inlineStr">
@@ -8799,13 +8799,13 @@
         <v>4.283</v>
       </c>
       <c r="L165" t="n">
-        <v>64.7</v>
+        <v>62.5</v>
       </c>
       <c r="M165" t="n">
         <v>4.127</v>
       </c>
       <c r="N165" t="n">
-        <v>37.3</v>
+        <v>35.4</v>
       </c>
       <c r="O165" t="inlineStr"/>
       <c r="P165" t="inlineStr">
@@ -8851,13 +8851,13 @@
         <v>4.308</v>
       </c>
       <c r="L166" t="n">
-        <v>71.09999999999999</v>
+        <v>69</v>
       </c>
       <c r="M166" t="n">
         <v>4.098</v>
       </c>
       <c r="N166" t="n">
-        <v>34.6</v>
+        <v>32.8</v>
       </c>
       <c r="O166" t="inlineStr"/>
       <c r="P166" t="inlineStr">
@@ -8903,13 +8903,13 @@
         <v>3.966</v>
       </c>
       <c r="L167" t="n">
-        <v>19.8</v>
+        <v>20</v>
       </c>
       <c r="M167" t="n">
         <v>3.432</v>
       </c>
       <c r="N167" t="n">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="O167" t="inlineStr"/>
       <c r="P167" t="inlineStr">
@@ -8955,13 +8955,13 @@
         <v>4.296</v>
       </c>
       <c r="L168" t="n">
-        <v>68.40000000000001</v>
+        <v>66.5</v>
       </c>
       <c r="M168" t="n">
         <v>4.169</v>
       </c>
       <c r="N168" t="n">
-        <v>42.2</v>
+        <v>39.9</v>
       </c>
       <c r="O168" t="inlineStr"/>
       <c r="P168" t="inlineStr">
@@ -9007,13 +9007,13 @@
         <v>4.02</v>
       </c>
       <c r="L169" t="n">
-        <v>24.6</v>
+        <v>24.5</v>
       </c>
       <c r="M169" t="n">
         <v>3.532</v>
       </c>
       <c r="N169" t="n">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="O169" t="inlineStr"/>
       <c r="P169" t="inlineStr">
@@ -9059,7 +9059,7 @@
         <v>4.314</v>
       </c>
       <c r="L170" t="n">
-        <v>73.3</v>
+        <v>71</v>
       </c>
       <c r="M170" t="n">
         <v>3.688</v>
@@ -9111,13 +9111,13 @@
         <v>4.268</v>
       </c>
       <c r="L171" t="n">
-        <v>60.4</v>
+        <v>58.5</v>
       </c>
       <c r="M171" t="n">
         <v>3.864</v>
       </c>
       <c r="N171" t="n">
-        <v>16.2</v>
+        <v>15.7</v>
       </c>
       <c r="O171" t="inlineStr"/>
       <c r="P171" t="inlineStr">
@@ -9163,7 +9163,7 @@
         <v>4.02</v>
       </c>
       <c r="L172" t="n">
-        <v>24.6</v>
+        <v>24.5</v>
       </c>
       <c r="M172" t="n">
         <v>3.602</v>
@@ -9215,13 +9215,13 @@
         <v>4.083</v>
       </c>
       <c r="L173" t="n">
-        <v>29.4</v>
+        <v>29</v>
       </c>
       <c r="M173" t="n">
         <v>3.554</v>
       </c>
       <c r="N173" t="n">
-        <v>4.3</v>
+        <v>4</v>
       </c>
       <c r="O173" t="inlineStr"/>
       <c r="P173" t="inlineStr">
@@ -9267,7 +9267,7 @@
         <v>3.93</v>
       </c>
       <c r="L174" t="n">
-        <v>16.6</v>
+        <v>17</v>
       </c>
       <c r="M174" t="n">
         <v>3.138</v>
@@ -9319,13 +9319,13 @@
         <v>3.93</v>
       </c>
       <c r="L175" t="n">
-        <v>16.6</v>
+        <v>17</v>
       </c>
       <c r="M175" t="n">
         <v>3.533</v>
       </c>
       <c r="N175" t="n">
-        <v>3.8</v>
+        <v>3.5</v>
       </c>
       <c r="O175" t="inlineStr"/>
       <c r="P175" t="inlineStr">
@@ -9371,13 +9371,13 @@
         <v>3.845</v>
       </c>
       <c r="L176" t="n">
-        <v>5.9</v>
+        <v>6.5</v>
       </c>
       <c r="M176" t="n">
         <v>3.445</v>
       </c>
       <c r="N176" t="n">
-        <v>2.2</v>
+        <v>2</v>
       </c>
       <c r="O176" t="inlineStr"/>
       <c r="P176" t="inlineStr">
@@ -9423,7 +9423,7 @@
         <v>3.897</v>
       </c>
       <c r="L177" t="n">
-        <v>14.4</v>
+        <v>14.5</v>
       </c>
       <c r="M177" t="n">
         <v>3.636</v>
@@ -9475,13 +9475,13 @@
         <v>4.264</v>
       </c>
       <c r="L178" t="n">
-        <v>57.2</v>
+        <v>55.5</v>
       </c>
       <c r="M178" t="n">
         <v>4.227</v>
       </c>
       <c r="N178" t="n">
-        <v>50.8</v>
+        <v>49</v>
       </c>
       <c r="O178" t="inlineStr"/>
       <c r="P178" t="inlineStr">
@@ -9527,13 +9527,13 @@
         <v>3.906</v>
       </c>
       <c r="L179" t="n">
-        <v>15</v>
+        <v>15.5</v>
       </c>
       <c r="M179" t="n">
         <v>3.751</v>
       </c>
       <c r="N179" t="n">
-        <v>10.8</v>
+        <v>10.6</v>
       </c>
       <c r="O179" t="inlineStr"/>
       <c r="P179" t="inlineStr">
@@ -9579,13 +9579,13 @@
         <v>3.973</v>
       </c>
       <c r="L180" t="n">
-        <v>20.3</v>
+        <v>20.5</v>
       </c>
       <c r="M180" t="n">
         <v>3.828</v>
       </c>
       <c r="N180" t="n">
-        <v>13.5</v>
+        <v>13.1</v>
       </c>
       <c r="O180" t="inlineStr"/>
       <c r="P180" t="inlineStr">
@@ -9631,13 +9631,13 @@
         <v>4.363</v>
       </c>
       <c r="L181" t="n">
-        <v>81.3</v>
+        <v>78.5</v>
       </c>
       <c r="M181" t="n">
         <v>4.632</v>
       </c>
       <c r="N181" t="n">
-        <v>94.59999999999999</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="O181" t="inlineStr"/>
       <c r="P181" t="inlineStr">
@@ -9683,13 +9683,13 @@
         <v>4.255</v>
       </c>
       <c r="L182" t="n">
-        <v>55.1</v>
+        <v>53.5</v>
       </c>
       <c r="M182" t="n">
         <v>4.351</v>
       </c>
       <c r="N182" t="n">
-        <v>64.90000000000001</v>
+        <v>62.1</v>
       </c>
       <c r="O182" t="inlineStr"/>
       <c r="P182" t="inlineStr">
@@ -9735,13 +9735,13 @@
         <v>4.264</v>
       </c>
       <c r="L183" t="n">
-        <v>57.2</v>
+        <v>55.5</v>
       </c>
       <c r="M183" t="n">
         <v>4.273</v>
       </c>
       <c r="N183" t="n">
-        <v>56.2</v>
+        <v>54</v>
       </c>
       <c r="O183" t="inlineStr"/>
       <c r="P183" t="inlineStr">
@@ -9787,13 +9787,13 @@
         <v>4.353</v>
       </c>
       <c r="L184" t="n">
-        <v>79.7</v>
+        <v>77</v>
       </c>
       <c r="M184" t="n">
         <v>4.24</v>
       </c>
       <c r="N184" t="n">
-        <v>52.4</v>
+        <v>50.5</v>
       </c>
       <c r="O184" t="inlineStr"/>
       <c r="P184" t="inlineStr">
@@ -9839,13 +9839,13 @@
         <v>4.218</v>
       </c>
       <c r="L185" t="n">
-        <v>48.7</v>
+        <v>47.5</v>
       </c>
       <c r="M185" t="n">
         <v>3.977</v>
       </c>
       <c r="N185" t="n">
-        <v>25.4</v>
+        <v>24.2</v>
       </c>
       <c r="O185" t="inlineStr"/>
       <c r="P185" t="inlineStr">
@@ -9891,13 +9891,13 @@
         <v>4.113</v>
       </c>
       <c r="L186" t="n">
-        <v>33.7</v>
+        <v>33</v>
       </c>
       <c r="M186" t="n">
         <v>4.639</v>
       </c>
       <c r="N186" t="n">
-        <v>95.09999999999999</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="O186" t="inlineStr"/>
       <c r="P186" t="inlineStr">
@@ -9943,13 +9943,13 @@
         <v>4.238</v>
       </c>
       <c r="L187" t="n">
-        <v>51.9</v>
+        <v>50.5</v>
       </c>
       <c r="M187" t="n">
         <v>4.561</v>
       </c>
       <c r="N187" t="n">
-        <v>90.3</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="O187" t="inlineStr"/>
       <c r="P187" t="inlineStr">
@@ -9995,13 +9995,13 @@
         <v>4.114</v>
       </c>
       <c r="L188" t="n">
-        <v>34.2</v>
+        <v>33.5</v>
       </c>
       <c r="M188" t="n">
         <v>4.33</v>
       </c>
       <c r="N188" t="n">
-        <v>62.2</v>
+        <v>59.6</v>
       </c>
       <c r="O188" t="inlineStr"/>
       <c r="P188" t="inlineStr">
@@ -10047,18 +10047,694 @@
         <v>3.865</v>
       </c>
       <c r="L189" t="n">
-        <v>7.5</v>
+        <v>8</v>
       </c>
       <c r="M189" t="n">
         <v>3.737</v>
       </c>
       <c r="N189" t="n">
-        <v>10.3</v>
+        <v>10.1</v>
       </c>
       <c r="O189" t="inlineStr"/>
       <c r="P189" t="inlineStr">
         <is>
           <t>Nigiri</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Wagyu Place</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Queens (Flushing)</t>
+        </is>
+      </c>
+      <c r="C190" t="n">
+        <v>68</v>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>varies (AYCE 90-120min)</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>AYCE wagyu yakiniku with complimentary omakase sushi set (A5 tier $159)</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr"/>
+      <c r="G190" t="inlineStr"/>
+      <c r="H190" t="inlineStr"/>
+      <c r="I190" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="J190" t="n">
+        <v>1686</v>
+      </c>
+      <c r="K190" t="n">
+        <v>4.394</v>
+      </c>
+      <c r="L190" t="n">
+        <v>83.5</v>
+      </c>
+      <c r="M190" t="n">
+        <v>4.567</v>
+      </c>
+      <c r="N190" t="n">
+        <v>86.40000000000001</v>
+      </c>
+      <c r="O190" t="inlineStr"/>
+      <c r="P190" t="inlineStr">
+        <is>
+          <t>Wagyu Place BBQ 和牛公馆</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Niku X NYC</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Manhattan (Midtown/Koreatown)</t>
+        </is>
+      </c>
+      <c r="C191" t="n">
+        <v>119</v>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>varies (AYCE 90-120min)</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Self-described 'only unlimited A5 Wagyu Steakhouse in the U.S.' with unlimited sushi+wagyu nigiri</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr"/>
+      <c r="G191" t="inlineStr"/>
+      <c r="H191" t="inlineStr"/>
+      <c r="I191" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="J191" t="n">
+        <v>2965</v>
+      </c>
+      <c r="K191" t="n">
+        <v>4.716</v>
+      </c>
+      <c r="L191" t="n">
+        <v>98.5</v>
+      </c>
+      <c r="M191" t="n">
+        <v>4.635</v>
+      </c>
+      <c r="N191" t="n">
+        <v>91.90000000000001</v>
+      </c>
+      <c r="O191" t="inlineStr"/>
+      <c r="P191" t="inlineStr">
+        <is>
+          <t>NIKU X | Limitless Wagyu BBQ &amp; Seafood</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Mikiya Wagyu Shabu House (Flushing)</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Queens (Flushing)</t>
+        </is>
+      </c>
+      <c r="C192" t="n">
+        <v>45</v>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>varies (AYCE 90-120min)</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>Shabu AYCE with A5 wagyu tiers; wagyu nigiri+tartare in every tier</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr"/>
+      <c r="G192" t="inlineStr"/>
+      <c r="H192" t="inlineStr"/>
+      <c r="I192" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="J192" t="n">
+        <v>1147</v>
+      </c>
+      <c r="K192" t="n">
+        <v>4.481</v>
+      </c>
+      <c r="L192" t="n">
+        <v>92.5</v>
+      </c>
+      <c r="M192" t="n">
+        <v>4.853</v>
+      </c>
+      <c r="N192" t="n">
+        <v>98</v>
+      </c>
+      <c r="O192" t="inlineStr"/>
+      <c r="P192" t="inlineStr">
+        <is>
+          <t>Mikiya Wagyu Shabu House 味喜屋 | Flushing</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Mikiya Wagyu Shabu House (Manhattan)</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Manhattan (Midtown East)</t>
+        </is>
+      </c>
+      <c r="C193" t="n">
+        <v>68</v>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>varies (AYCE 90-120min)</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Manhattan sister of Mikiya Flushing; explicit AYCE wagyu nigiri program</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr"/>
+      <c r="G193" t="inlineStr"/>
+      <c r="H193" t="inlineStr"/>
+      <c r="I193" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="J193" t="n">
+        <v>345</v>
+      </c>
+      <c r="K193" t="n">
+        <v>4.409</v>
+      </c>
+      <c r="L193" t="n">
+        <v>85.5</v>
+      </c>
+      <c r="M193" t="n">
+        <v>4.582</v>
+      </c>
+      <c r="N193" t="n">
+        <v>87.40000000000001</v>
+      </c>
+      <c r="O193" t="inlineStr"/>
+      <c r="P193" t="inlineStr">
+        <is>
+          <t>Mikiya Wagyu Shabu House | Manhattan</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Chubby Cattle BBQ NYC</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Manhattan (SoHo)</t>
+        </is>
+      </c>
+      <c r="C194" t="n">
+        <v>58</v>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>varies (AYCE 90-120min)</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>Signature Wagyu Uni Caviar Nigiri served as part of AYCE wagyu yakiniku</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr"/>
+      <c r="G194" t="inlineStr"/>
+      <c r="H194" t="inlineStr"/>
+      <c r="I194" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="J194" t="n">
+        <v>2382</v>
+      </c>
+      <c r="K194" t="n">
+        <v>4.711</v>
+      </c>
+      <c r="L194" t="n">
+        <v>98</v>
+      </c>
+      <c r="M194" t="n">
+        <v>4.975</v>
+      </c>
+      <c r="N194" t="n">
+        <v>99.5</v>
+      </c>
+      <c r="O194" t="inlineStr"/>
+      <c r="P194" t="inlineStr">
+        <is>
+          <t>Chubby Cattle BBQ | New York</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Y Space BBQ</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Queens (Flushing)</t>
+        </is>
+      </c>
+      <c r="C195" t="n">
+        <v>49</v>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>varies (AYCE 90-120min)</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>Space-themed AYCE wagyu yakiniku with A5 Wagyu Nigiri Sushi as part of AYCE</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr"/>
+      <c r="G195" t="inlineStr"/>
+      <c r="H195" t="inlineStr"/>
+      <c r="I195" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="J195" t="n">
+        <v>1559</v>
+      </c>
+      <c r="K195" t="n">
+        <v>4.289</v>
+      </c>
+      <c r="L195" t="n">
+        <v>64.5</v>
+      </c>
+      <c r="M195" t="n">
+        <v>4.606</v>
+      </c>
+      <c r="N195" t="n">
+        <v>88.90000000000001</v>
+      </c>
+      <c r="O195" t="inlineStr"/>
+      <c r="P195" t="inlineStr">
+        <is>
+          <t>Y Space BBQ 烤肉火焱星</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Wagyu Yama Yakiniku &amp; Seafood Shabu</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Queens (Flushing)</t>
+        </is>
+      </c>
+      <c r="C196" t="n">
+        <v>68</v>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>varies (AYCE 90-120min)</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>A5 yakiniku + seafood shabu hybrid; AYCE BBQ + hotpot combo with sashimi rounds</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr"/>
+      <c r="G196" t="inlineStr"/>
+      <c r="H196" t="inlineStr"/>
+      <c r="I196" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="J196" t="n">
+        <v>1147</v>
+      </c>
+      <c r="K196" t="n">
+        <v>4.481</v>
+      </c>
+      <c r="L196" t="n">
+        <v>92.5</v>
+      </c>
+      <c r="M196" t="n">
+        <v>4.657</v>
+      </c>
+      <c r="N196" t="n">
+        <v>93.90000000000001</v>
+      </c>
+      <c r="O196" t="inlineStr"/>
+      <c r="P196" t="inlineStr">
+        <is>
+          <t>Mikiya Wagyu Shabu House 味喜屋 | Flushing</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Hiyake Omakase (Bowery)</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Manhattan (Lower East Side/Chinatown)</t>
+        </is>
+      </c>
+      <c r="C197" t="n">
+        <v>29</v>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>varies (AYCE 90-120min)</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>AYCE wagyu yakiniku with Uni Wagyu Handroll; despite the name, it's not counter omakase</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr"/>
+      <c r="G197" t="inlineStr"/>
+      <c r="H197" t="inlineStr"/>
+      <c r="I197" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="J197" t="n">
+        <v>98</v>
+      </c>
+      <c r="K197" t="n">
+        <v>4.367</v>
+      </c>
+      <c r="L197" t="n">
+        <v>79</v>
+      </c>
+      <c r="M197" t="n">
+        <v>4.942</v>
+      </c>
+      <c r="N197" t="n">
+        <v>99</v>
+      </c>
+      <c r="O197" t="inlineStr"/>
+      <c r="P197" t="inlineStr">
+        <is>
+          <t>Genki east omakase</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>Hiyake Omakase (Williamsburg)</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Brooklyn (Williamsburg)</t>
+        </is>
+      </c>
+      <c r="C198" t="n">
+        <v>48</v>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>varies (AYCE 90-120min)</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>Brooklyn sister of Hiyake; AYCE wagyu yakiniku with sushi+sashimi rounds in private booths</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr"/>
+      <c r="G198" t="inlineStr"/>
+      <c r="H198" t="inlineStr"/>
+      <c r="I198" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="J198" t="n">
+        <v>171</v>
+      </c>
+      <c r="K198" t="n">
+        <v>3.904</v>
+      </c>
+      <c r="L198" t="n">
+        <v>15</v>
+      </c>
+      <c r="M198" t="n">
+        <v>4.201</v>
+      </c>
+      <c r="N198" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="O198" t="inlineStr"/>
+      <c r="P198" t="inlineStr">
+        <is>
+          <t>Hiyake Yakiniku BBQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Gyu-Ichiro</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Manhattan (Lower East Side/Chinatown)</t>
+        </is>
+      </c>
+      <c r="C199" t="n">
+        <v>29</v>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>varies (AYCE 90-120min)</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>Same operator/space as Hiyake; markets unlimited wagyu + sushi combo</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr"/>
+      <c r="G199" t="inlineStr"/>
+      <c r="H199" t="inlineStr"/>
+      <c r="I199" t="n">
+        <v>4</v>
+      </c>
+      <c r="J199" t="n">
+        <v>353</v>
+      </c>
+      <c r="K199" t="n">
+        <v>3.684</v>
+      </c>
+      <c r="L199" t="n">
+        <v>3</v>
+      </c>
+      <c r="M199" t="n">
+        <v>4.169</v>
+      </c>
+      <c r="N199" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="O199" t="inlineStr"/>
+      <c r="P199" t="inlineStr">
+        <is>
+          <t>Gyu-Ichiro Japanese BBQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Nikushou Sakai</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Queens (Flushing)</t>
+        </is>
+      </c>
+      <c r="C200" t="n">
+        <v>55</v>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>varies (AYCE 90-120min)</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>New 2025 Flushing AYCE wagyu yakiniku with sashimi inclusion (iPad ordering)</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr"/>
+      <c r="G200" t="inlineStr"/>
+      <c r="H200" t="inlineStr"/>
+      <c r="I200" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="J200" t="n">
+        <v>264</v>
+      </c>
+      <c r="K200" t="n">
+        <v>3.351</v>
+      </c>
+      <c r="L200" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M200" t="n">
+        <v>3.557</v>
+      </c>
+      <c r="N200" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="O200" t="inlineStr"/>
+      <c r="P200" t="inlineStr">
+        <is>
+          <t>Nikushou Sakai 肉匠坂井</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Umiya Sushi LIC</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Queens (Long Island City)</t>
+        </is>
+      </c>
+      <c r="C201" t="n">
+        <v>40</v>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>varies (AYCE 90-120min)</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>AYCE sushi bar with A5 Japanese Wagyu in Premium tier ($67.95)</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr"/>
+      <c r="G201" t="inlineStr"/>
+      <c r="H201" t="inlineStr"/>
+      <c r="I201" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="J201" t="n">
+        <v>482</v>
+      </c>
+      <c r="K201" t="n">
+        <v>4.435</v>
+      </c>
+      <c r="L201" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="M201" t="n">
+        <v>4.861</v>
+      </c>
+      <c r="N201" t="n">
+        <v>98.5</v>
+      </c>
+      <c r="O201" t="inlineStr"/>
+      <c r="P201" t="inlineStr">
+        <is>
+          <t>Umiya Sushi</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Asuka Sushi</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Manhattan (Chelsea)</t>
+        </is>
+      </c>
+      <c r="C202" t="n">
+        <v>30</v>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>varies (AYCE 90-120min)</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>Chelsea sushi bar with signature Big Mac (wagyu+uni+scallop+toro) and AYCE wagyu sushi</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr"/>
+      <c r="G202" t="inlineStr"/>
+      <c r="H202" t="inlineStr"/>
+      <c r="I202" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="J202" t="n">
+        <v>1436</v>
+      </c>
+      <c r="K202" t="n">
+        <v>4.185</v>
+      </c>
+      <c r="L202" t="n">
+        <v>44</v>
+      </c>
+      <c r="M202" t="n">
+        <v>4.72</v>
+      </c>
+      <c r="N202" t="n">
+        <v>95.5</v>
+      </c>
+      <c r="O202" t="inlineStr"/>
+      <c r="P202" t="inlineStr">
+        <is>
+          <t>Asuka Sushi</t>
         </is>
       </c>
     </row>

</xml_diff>